<commit_message>
fix(finance): follow up fixes for local storage, UUID API errors, PDF styles, and cash flow sorting
</commit_message>
<xml_diff>
--- a/references/CATATAN KEUANGAN PADI 1 Ha ADE.xlsx
+++ b/references/CATATAN KEUANGAN PADI 1 Ha ADE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\My Files\Projects\arina-agri\references\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DEF85D8-6705-45AA-A7CE-6C949572664A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1E54F33-783F-4177-8707-AFD165EA84E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-45" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-45" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. RAB PADI 1 Ha" sheetId="9" r:id="rId1"/>
@@ -2338,6 +2338,60 @@
     <xf numFmtId="170" fontId="2" fillId="0" borderId="16" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="172" fontId="2" fillId="0" borderId="74" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="2" fillId="0" borderId="75" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="65" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="66" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="0" fillId="0" borderId="42" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="0" fillId="0" borderId="78" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="0" fillId="0" borderId="80" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="0" fillId="0" borderId="81" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="2" fillId="0" borderId="42" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="2" fillId="0" borderId="78" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="70" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="71" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="0" fillId="0" borderId="72" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="0" fillId="0" borderId="73" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="72" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="73" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="72" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="73" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="170" fontId="2" fillId="0" borderId="15" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2367,12 +2421,6 @@
     </xf>
     <xf numFmtId="170" fontId="9" fillId="8" borderId="14" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="65" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="66" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="62" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2409,54 +2457,6 @@
     </xf>
     <xf numFmtId="170" fontId="16" fillId="6" borderId="17" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="2" fillId="0" borderId="42" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="2" fillId="0" borderId="78" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="70" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="71" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="175" fontId="0" fillId="0" borderId="72" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="175" fontId="0" fillId="0" borderId="73" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="72" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="73" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="72" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="73" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="2" fillId="0" borderId="74" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="2" fillId="0" borderId="75" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="175" fontId="0" fillId="0" borderId="42" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="175" fontId="0" fillId="0" borderId="78" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="175" fontId="0" fillId="0" borderId="80" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="175" fontId="0" fillId="0" borderId="81" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -10941,30 +10941,30 @@
     <row r="3" spans="2:17" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="157"/>
       <c r="C3" s="158"/>
-      <c r="D3" s="258" t="s">
+      <c r="D3" s="276" t="s">
         <v>167</v>
       </c>
-      <c r="E3" s="259"/>
-      <c r="F3" s="259"/>
-      <c r="G3" s="259"/>
-      <c r="H3" s="259"/>
-      <c r="I3" s="259"/>
-      <c r="J3" s="259"/>
-      <c r="K3" s="260"/>
+      <c r="E3" s="277"/>
+      <c r="F3" s="277"/>
+      <c r="G3" s="277"/>
+      <c r="H3" s="277"/>
+      <c r="I3" s="277"/>
+      <c r="J3" s="277"/>
+      <c r="K3" s="278"/>
       <c r="L3" s="158"/>
       <c r="M3" s="159"/>
     </row>
     <row r="4" spans="2:17" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="157"/>
       <c r="C4" s="158"/>
-      <c r="D4" s="261"/>
-      <c r="E4" s="262"/>
-      <c r="F4" s="262"/>
-      <c r="G4" s="262"/>
-      <c r="H4" s="262"/>
-      <c r="I4" s="262"/>
-      <c r="J4" s="262"/>
-      <c r="K4" s="263"/>
+      <c r="D4" s="279"/>
+      <c r="E4" s="280"/>
+      <c r="F4" s="280"/>
+      <c r="G4" s="280"/>
+      <c r="H4" s="280"/>
+      <c r="I4" s="280"/>
+      <c r="J4" s="280"/>
+      <c r="K4" s="281"/>
       <c r="L4" s="158"/>
       <c r="M4" s="159"/>
     </row>
@@ -11002,14 +11002,14 @@
     </row>
     <row r="7" spans="2:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="157"/>
-      <c r="C7" s="254" t="s">
+      <c r="C7" s="272" t="s">
         <v>152</v>
       </c>
-      <c r="D7" s="255"/>
-      <c r="E7" s="256" t="s">
+      <c r="D7" s="273"/>
+      <c r="E7" s="274" t="s">
         <v>153</v>
       </c>
-      <c r="F7" s="257"/>
+      <c r="F7" s="275"/>
       <c r="G7" s="167" t="s">
         <v>154</v>
       </c>
@@ -11034,8 +11034,8 @@
       <c r="B8" s="157"/>
       <c r="C8" s="169"/>
       <c r="D8" s="158"/>
-      <c r="E8" s="264"/>
-      <c r="F8" s="265"/>
+      <c r="E8" s="256"/>
+      <c r="F8" s="257"/>
       <c r="G8" s="170"/>
       <c r="H8" s="170"/>
       <c r="I8" s="170"/>
@@ -11050,8 +11050,8 @@
         <v>169</v>
       </c>
       <c r="D9" s="158"/>
-      <c r="E9" s="266"/>
-      <c r="F9" s="267"/>
+      <c r="E9" s="282"/>
+      <c r="F9" s="283"/>
       <c r="G9" s="141">
         <f>'4. Arus kas'!G44</f>
         <v>-13464000</v>
@@ -11110,13 +11110,13 @@
       <c r="B12" s="157"/>
       <c r="C12" s="178"/>
       <c r="D12" s="158"/>
-      <c r="E12" s="268" t="s">
+      <c r="E12" s="284" t="s">
         <v>170</v>
       </c>
-      <c r="F12" s="269"/>
-      <c r="G12" s="269"/>
-      <c r="H12" s="269"/>
-      <c r="I12" s="269"/>
+      <c r="F12" s="285"/>
+      <c r="G12" s="285"/>
+      <c r="H12" s="285"/>
+      <c r="I12" s="285"/>
       <c r="J12" s="179"/>
       <c r="K12" s="158"/>
       <c r="L12" s="152"/>
@@ -11128,12 +11128,12 @@
       <c r="B13" s="157"/>
       <c r="C13" s="178"/>
       <c r="D13" s="158"/>
-      <c r="E13" s="270" t="s">
+      <c r="E13" s="286" t="s">
         <v>152</v>
       </c>
-      <c r="F13" s="271"/>
-      <c r="G13" s="271"/>
-      <c r="H13" s="271"/>
+      <c r="F13" s="287"/>
+      <c r="G13" s="287"/>
+      <c r="H13" s="287"/>
       <c r="I13" s="168" t="s">
         <v>159</v>
       </c>
@@ -11230,11 +11230,11 @@
       <c r="C18" s="178"/>
       <c r="D18" s="158"/>
       <c r="E18" s="169"/>
-      <c r="F18" s="272" t="s">
+      <c r="F18" s="288" t="s">
         <v>173</v>
       </c>
-      <c r="G18" s="272"/>
-      <c r="H18" s="272"/>
+      <c r="G18" s="288"/>
+      <c r="H18" s="288"/>
       <c r="I18" s="184">
         <f>I15-I16</f>
         <v>15000000</v>
@@ -11361,11 +11361,11 @@
       <c r="C25" s="178"/>
       <c r="D25" s="158"/>
       <c r="E25" s="169"/>
-      <c r="F25" s="273" t="s">
+      <c r="F25" s="289" t="s">
         <v>178</v>
       </c>
-      <c r="G25" s="273"/>
-      <c r="H25" s="274"/>
+      <c r="G25" s="289"/>
+      <c r="H25" s="290"/>
       <c r="I25" s="195">
         <f>I18*3%</f>
         <v>450000</v>
@@ -11382,11 +11382,11 @@
       <c r="C26" s="178"/>
       <c r="D26" s="158"/>
       <c r="E26" s="169"/>
-      <c r="F26" s="272" t="s">
+      <c r="F26" s="288" t="s">
         <v>179</v>
       </c>
-      <c r="G26" s="272"/>
-      <c r="H26" s="272"/>
+      <c r="G26" s="288"/>
+      <c r="H26" s="288"/>
       <c r="I26" s="184">
         <f>I18+I25</f>
         <v>15450000</v>
@@ -11430,32 +11430,32 @@
     </row>
     <row r="29" spans="2:15" s="166" customFormat="1" ht="29.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B29" s="160"/>
-      <c r="C29" s="275" t="s">
+      <c r="C29" s="291" t="s">
         <v>180</v>
       </c>
-      <c r="D29" s="276"/>
-      <c r="E29" s="276"/>
-      <c r="F29" s="276"/>
-      <c r="G29" s="276"/>
-      <c r="H29" s="276"/>
-      <c r="I29" s="276"/>
-      <c r="J29" s="276"/>
-      <c r="K29" s="276"/>
-      <c r="L29" s="277"/>
+      <c r="D29" s="292"/>
+      <c r="E29" s="292"/>
+      <c r="F29" s="292"/>
+      <c r="G29" s="292"/>
+      <c r="H29" s="292"/>
+      <c r="I29" s="292"/>
+      <c r="J29" s="292"/>
+      <c r="K29" s="292"/>
+      <c r="L29" s="293"/>
       <c r="M29" s="164"/>
       <c r="N29" s="165"/>
       <c r="O29" s="165"/>
     </row>
     <row r="30" spans="2:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B30" s="157"/>
-      <c r="C30" s="254" t="s">
+      <c r="C30" s="272" t="s">
         <v>152</v>
       </c>
-      <c r="D30" s="255"/>
-      <c r="E30" s="256" t="s">
+      <c r="D30" s="273"/>
+      <c r="E30" s="274" t="s">
         <v>153</v>
       </c>
-      <c r="F30" s="257"/>
+      <c r="F30" s="275"/>
       <c r="G30" s="167" t="s">
         <v>154</v>
       </c>
@@ -11482,8 +11482,8 @@
         <v>181</v>
       </c>
       <c r="D31" s="158"/>
-      <c r="E31" s="264"/>
-      <c r="F31" s="265"/>
+      <c r="E31" s="256"/>
+      <c r="F31" s="257"/>
       <c r="G31" s="170"/>
       <c r="H31" s="170"/>
       <c r="I31" s="170"/>
@@ -11498,11 +11498,11 @@
       <c r="D32" s="158" t="s">
         <v>172</v>
       </c>
-      <c r="E32" s="280">
+      <c r="E32" s="264">
         <f>I16</f>
         <v>3869000</v>
       </c>
-      <c r="F32" s="281"/>
+      <c r="F32" s="265"/>
       <c r="G32" s="198"/>
       <c r="H32" s="198"/>
       <c r="I32" s="198"/>
@@ -11520,11 +11520,11 @@
       <c r="D33" s="158" t="s">
         <v>182</v>
       </c>
-      <c r="E33" s="282">
+      <c r="E33" s="266">
         <f>I18</f>
         <v>15000000</v>
       </c>
-      <c r="F33" s="283"/>
+      <c r="F33" s="267"/>
       <c r="G33" s="199"/>
       <c r="H33" s="199"/>
       <c r="I33" s="199"/>
@@ -11546,8 +11546,8 @@
       <c r="D34" s="158" t="s">
         <v>183</v>
       </c>
-      <c r="E34" s="284"/>
-      <c r="F34" s="285"/>
+      <c r="E34" s="268"/>
+      <c r="F34" s="269"/>
       <c r="G34" s="201"/>
       <c r="H34" s="201"/>
       <c r="I34" s="201"/>
@@ -11566,8 +11566,8 @@
       <c r="B35" s="157"/>
       <c r="C35" s="169"/>
       <c r="D35" s="158"/>
-      <c r="E35" s="286"/>
-      <c r="F35" s="287"/>
+      <c r="E35" s="270"/>
+      <c r="F35" s="271"/>
       <c r="G35" s="201"/>
       <c r="H35" s="201"/>
       <c r="I35" s="201"/>
@@ -11585,21 +11585,21 @@
       <c r="D36" s="203" t="s">
         <v>181</v>
       </c>
-      <c r="E36" s="288">
+      <c r="E36" s="254">
         <f>SUM(E32:F35)</f>
         <v>18869000</v>
       </c>
-      <c r="F36" s="289"/>
-      <c r="G36" s="288">
+      <c r="F36" s="255"/>
+      <c r="G36" s="254">
         <f t="shared" ref="G36" si="0">SUM(G32:H35)</f>
         <v>0</v>
       </c>
-      <c r="H36" s="289"/>
-      <c r="I36" s="288">
+      <c r="H36" s="255"/>
+      <c r="I36" s="254">
         <f t="shared" ref="I36" si="1">SUM(I32:J35)</f>
         <v>0</v>
       </c>
-      <c r="J36" s="289"/>
+      <c r="J36" s="255"/>
       <c r="K36" s="204">
         <f t="shared" ref="K36" si="2">SUM(K32:K34)</f>
         <v>-15450000</v>
@@ -11611,8 +11611,8 @@
       <c r="B37" s="157"/>
       <c r="C37" s="169"/>
       <c r="D37" s="158"/>
-      <c r="E37" s="264"/>
-      <c r="F37" s="265"/>
+      <c r="E37" s="256"/>
+      <c r="F37" s="257"/>
       <c r="G37" s="170"/>
       <c r="H37" s="170"/>
       <c r="I37" s="170"/>
@@ -11627,11 +11627,11 @@
       <c r="D38" s="206" t="s">
         <v>184</v>
       </c>
-      <c r="E38" s="290">
+      <c r="E38" s="258">
         <f>E9</f>
         <v>0</v>
       </c>
-      <c r="F38" s="291"/>
+      <c r="F38" s="259"/>
       <c r="G38" s="207">
         <f>G9</f>
         <v>-13464000</v>
@@ -11663,8 +11663,8 @@
       <c r="B39" s="157"/>
       <c r="C39" s="169"/>
       <c r="D39" s="158"/>
-      <c r="E39" s="292"/>
-      <c r="F39" s="293"/>
+      <c r="E39" s="260"/>
+      <c r="F39" s="261"/>
       <c r="G39" s="211"/>
       <c r="H39" s="212"/>
       <c r="I39" s="212"/>
@@ -11679,11 +11679,11 @@
       <c r="D40" s="214" t="s">
         <v>185</v>
       </c>
-      <c r="E40" s="278">
+      <c r="E40" s="262">
         <f>E36+E38</f>
         <v>18869000</v>
       </c>
-      <c r="F40" s="279"/>
+      <c r="F40" s="263"/>
       <c r="G40" s="208">
         <f>E40+G38</f>
         <v>5405000</v>
@@ -11746,18 +11746,6 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="G36:H36"/>
-    <mergeCell ref="I36:J36"/>
-    <mergeCell ref="E37:F37"/>
-    <mergeCell ref="E38:F38"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="E32:F32"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="E36:F36"/>
     <mergeCell ref="C30:D30"/>
     <mergeCell ref="E30:F30"/>
     <mergeCell ref="D3:K4"/>
@@ -11771,6 +11759,18 @@
     <mergeCell ref="F25:H25"/>
     <mergeCell ref="F26:H26"/>
     <mergeCell ref="C29:L29"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="I36:J36"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="E39:F39"/>
   </mergeCells>
   <pageMargins left="0.5" right="0" top="0.49803149600000002" bottom="0" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="75" orientation="landscape" r:id="rId1"/>

</xml_diff>